<commit_message>
Update links to use custom domain
</commit_message>
<xml_diff>
--- a/assets/planilha_mestra_cultivo.xlsx
+++ b/assets/planilha_mestra_cultivo.xlsx
@@ -1,18 +1,23 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <fileVersion rupBuild="9303" lowestEdited="5" lastEdited="5" appName="xl"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
+  <fileVersion appName="xl" lastEdited="6" lowestEdited="5" rupBuild="14420"/>
   <workbookPr/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Projetos\ZHC\website\assets\"/>
+    </mc:Choice>
+  </mc:AlternateContent>
   <bookViews>
-    <workbookView xWindow="480" yWindow="60" windowWidth="18195" windowHeight="8505" activeTab="2"/>
+    <workbookView xWindow="480" yWindow="60" windowWidth="18192" windowHeight="8508"/>
   </bookViews>
   <sheets>
-    <sheet r:id="rId1" sheetId="1" name="Configuração Inicial"/>
-    <sheet r:id="rId2" sheetId="2" name="Diário Semanal"/>
-    <sheet r:id="rId3" sheetId="3" name="Manejo Orgânico (IPM)"/>
-    <sheet r:id="rId4" sheetId="4" name="Database"/>
+    <sheet name="Configuração Inicial" sheetId="1" r:id="rId1"/>
+    <sheet name="Diário Semanal" sheetId="2" r:id="rId2"/>
+    <sheet name="Manejo Orgânico (IPM)" sheetId="3" r:id="rId3"/>
+    <sheet name="Database" sheetId="4" r:id="rId4"/>
   </sheets>
-  <calcPr fullCalcOnLoad="1"/>
+  <calcPr calcId="162913"/>
 </workbook>
 </file>
 
@@ -184,10 +189,7 @@
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" mc:Ignorable="x14ac">
-  <numFmts count="1">
-    <numFmt numFmtId="164" formatCode="dd/mm/yyyy"/>
-  </numFmts>
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
   <fonts count="5" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
@@ -199,7 +201,7 @@
     <font>
       <b/>
       <sz val="11"/>
-      <color rgb="FFffffff"/>
+      <color rgb="FFFFFFFF"/>
       <name val="Calibri"/>
       <family val="2"/>
     </font>
@@ -232,17 +234,17 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FF2e7d32"/>
+        <fgColor rgb="FF2E7D32"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFf5f5f5"/>
+        <fgColor rgb="FFF5F5F5"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFe8f5e9"/>
+        <fgColor rgb="FFE8F5E9"/>
       </patternFill>
     </fill>
   </fills>
@@ -280,53 +282,58 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="13">
-    <xf xfId="0" numFmtId="0" borderId="0" fontId="0" fillId="0"/>
-    <xf xfId="0" numFmtId="0" borderId="0" fontId="0" fillId="0" applyAlignment="1">
-      <alignment horizontal="general"/>
-    </xf>
-    <xf xfId="0" numFmtId="0" borderId="0" fontId="0" fillId="0" applyAlignment="1">
-      <alignment horizontal="general"/>
-    </xf>
-    <xf xfId="0" numFmtId="0" borderId="1" applyBorder="1" fontId="1" applyFont="1" fillId="2" applyFill="1" applyAlignment="1">
+  <cellXfs count="15">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="1" applyBorder="1" fontId="1" applyFont="1" fillId="2" applyFill="1" applyAlignment="1">
+    <xf numFmtId="3" fontId="1" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="1" applyBorder="1" fontId="2" applyFont="1" fillId="3" applyFill="1" applyAlignment="1">
+    <xf numFmtId="3" fontId="2" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="0" fontId="0" fillId="0" applyAlignment="1">
+    <xf numFmtId="3" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf xfId="0" numFmtId="164" applyNumberFormat="1" borderId="1" applyBorder="1" fontId="3" applyFont="1" fillId="0" applyAlignment="1">
+    <xf numFmtId="14" fontId="3" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="2" applyBorder="1" fontId="3" applyFont="1" fillId="0" applyAlignment="1">
+    <xf numFmtId="3" fontId="3" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf xfId="0" numFmtId="0" borderId="0" fontId="0" fillId="0" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="0" fontId="0" fillId="0" applyAlignment="1">
+    <xf numFmtId="3" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="1" applyBorder="1" fontId="4" applyFont="1" fillId="4" applyFill="1" applyAlignment="1">
+    <xf numFmtId="3" fontId="4" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="0" fontId="0" fillId="0" applyAlignment="1">
+    <xf numFmtId="3" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="1" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle xfId="0" builtinId="0" name="Normal"/>
+    <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
   <extLst>
-    <ext uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
-      <x14ac:slicerStyles xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" defaultSlicerStyle="SlicerStyleLight1"/>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
+      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
+    </ext>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
+      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
     </ext>
   </extLst>
 </styleSheet>
@@ -337,10 +344,10 @@
   <a:themeElements>
     <a:clrScheme name="Office">
       <a:dk1>
-        <a:sysClr lastClr="000000" val="windowText"/>
+        <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
       <a:lt1>
-        <a:sysClr lastClr="FFFFFF" val="window"/>
+        <a:sysClr val="window" lastClr="FFFFFF"/>
       </a:lt1>
       <a:dk2>
         <a:srgbClr val="1F497D"/>
@@ -378,71 +385,71 @@
         <a:latin typeface="Cambria"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
-        <a:font typeface="ＭＳ Ｐゴシック" script="Jpan"/>
-        <a:font typeface="맑은 고딕" script="Hang"/>
-        <a:font typeface="宋体" script="Hans"/>
-        <a:font typeface="新細明體" script="Hant"/>
-        <a:font typeface="Times New Roman" script="Arab"/>
-        <a:font typeface="Times New Roman" script="Hebr"/>
-        <a:font typeface="Tahoma" script="Thai"/>
-        <a:font typeface="Nyala" script="Ethi"/>
-        <a:font typeface="Vrinda" script="Beng"/>
-        <a:font typeface="Shruti" script="Gujr"/>
-        <a:font typeface="MoolBoran" script="Khmr"/>
-        <a:font typeface="Tunga" script="Knda"/>
-        <a:font typeface="Raavi" script="Guru"/>
-        <a:font typeface="Euphemia" script="Cans"/>
-        <a:font typeface="Plantagenet Cherokee" script="Cher"/>
-        <a:font typeface="Microsoft Yi Baiti" script="Yiii"/>
-        <a:font typeface="Microsoft Himalaya" script="Tibt"/>
-        <a:font typeface="MV Boli" script="Thaa"/>
-        <a:font typeface="Mangal" script="Deva"/>
-        <a:font typeface="Gautami" script="Telu"/>
-        <a:font typeface="Latha" script="Taml"/>
-        <a:font typeface="Estrangelo Edessa" script="Syrc"/>
-        <a:font typeface="Kalinga" script="Orya"/>
-        <a:font typeface="Kartika" script="Mlym"/>
-        <a:font typeface="DokChampa" script="Laoo"/>
-        <a:font typeface="Iskoola Pota" script="Sinh"/>
-        <a:font typeface="Mongolian Baiti" script="Mong"/>
-        <a:font typeface="Times New Roman" script="Viet"/>
-        <a:font typeface="Microsoft Uighur" script="Uigh"/>
-        <a:font typeface="Sylfaen" script="Geor"/>
+        <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
+        <a:font script="Hang" typeface="맑은 고딕"/>
+        <a:font script="Hans" typeface="宋体"/>
+        <a:font script="Hant" typeface="新細明體"/>
+        <a:font script="Arab" typeface="Times New Roman"/>
+        <a:font script="Hebr" typeface="Times New Roman"/>
+        <a:font script="Thai" typeface="Tahoma"/>
+        <a:font script="Ethi" typeface="Nyala"/>
+        <a:font script="Beng" typeface="Vrinda"/>
+        <a:font script="Gujr" typeface="Shruti"/>
+        <a:font script="Khmr" typeface="MoolBoran"/>
+        <a:font script="Knda" typeface="Tunga"/>
+        <a:font script="Guru" typeface="Raavi"/>
+        <a:font script="Cans" typeface="Euphemia"/>
+        <a:font script="Cher" typeface="Plantagenet Cherokee"/>
+        <a:font script="Yiii" typeface="Microsoft Yi Baiti"/>
+        <a:font script="Tibt" typeface="Microsoft Himalaya"/>
+        <a:font script="Thaa" typeface="MV Boli"/>
+        <a:font script="Deva" typeface="Mangal"/>
+        <a:font script="Telu" typeface="Gautami"/>
+        <a:font script="Taml" typeface="Latha"/>
+        <a:font script="Syrc" typeface="Estrangelo Edessa"/>
+        <a:font script="Orya" typeface="Kalinga"/>
+        <a:font script="Mlym" typeface="Kartika"/>
+        <a:font script="Laoo" typeface="DokChampa"/>
+        <a:font script="Sinh" typeface="Iskoola Pota"/>
+        <a:font script="Mong" typeface="Mongolian Baiti"/>
+        <a:font script="Viet" typeface="Times New Roman"/>
+        <a:font script="Uigh" typeface="Microsoft Uighur"/>
+        <a:font script="Geor" typeface="Sylfaen"/>
       </a:majorFont>
       <a:minorFont>
         <a:latin typeface="Calibri"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
-        <a:font typeface="ＭＳ Ｐゴシック" script="Jpan"/>
-        <a:font typeface="맑은 고딕" script="Hang"/>
-        <a:font typeface="宋体" script="Hans"/>
-        <a:font typeface="新細明體" script="Hant"/>
-        <a:font typeface="Arial" script="Arab"/>
-        <a:font typeface="Arial" script="Hebr"/>
-        <a:font typeface="Tahoma" script="Thai"/>
-        <a:font typeface="Nyala" script="Ethi"/>
-        <a:font typeface="Vrinda" script="Beng"/>
-        <a:font typeface="Shruti" script="Gujr"/>
-        <a:font typeface="DaunPenh" script="Khmr"/>
-        <a:font typeface="Tunga" script="Knda"/>
-        <a:font typeface="Raavi" script="Guru"/>
-        <a:font typeface="Euphemia" script="Cans"/>
-        <a:font typeface="Plantagenet Cherokee" script="Cher"/>
-        <a:font typeface="Microsoft Yi Baiti" script="Yiii"/>
-        <a:font typeface="Microsoft Himalaya" script="Tibt"/>
-        <a:font typeface="MV Boli" script="Thaa"/>
-        <a:font typeface="Mangal" script="Deva"/>
-        <a:font typeface="Gautami" script="Telu"/>
-        <a:font typeface="Latha" script="Taml"/>
-        <a:font typeface="Estrangelo Edessa" script="Syrc"/>
-        <a:font typeface="Kalinga" script="Orya"/>
-        <a:font typeface="Kartika" script="Mlym"/>
-        <a:font typeface="DokChampa" script="Laoo"/>
-        <a:font typeface="Iskoola Pota" script="Sinh"/>
-        <a:font typeface="Mongolian Baiti" script="Mong"/>
-        <a:font typeface="Arial" script="Viet"/>
-        <a:font typeface="Microsoft Uighur" script="Uigh"/>
-        <a:font typeface="Sylfaen" script="Geor"/>
+        <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
+        <a:font script="Hang" typeface="맑은 고딕"/>
+        <a:font script="Hans" typeface="宋体"/>
+        <a:font script="Hant" typeface="新細明體"/>
+        <a:font script="Arab" typeface="Arial"/>
+        <a:font script="Hebr" typeface="Arial"/>
+        <a:font script="Thai" typeface="Tahoma"/>
+        <a:font script="Ethi" typeface="Nyala"/>
+        <a:font script="Beng" typeface="Vrinda"/>
+        <a:font script="Gujr" typeface="Shruti"/>
+        <a:font script="Khmr" typeface="DaunPenh"/>
+        <a:font script="Knda" typeface="Tunga"/>
+        <a:font script="Guru" typeface="Raavi"/>
+        <a:font script="Cans" typeface="Euphemia"/>
+        <a:font script="Cher" typeface="Plantagenet Cherokee"/>
+        <a:font script="Yiii" typeface="Microsoft Yi Baiti"/>
+        <a:font script="Tibt" typeface="Microsoft Himalaya"/>
+        <a:font script="Thaa" typeface="MV Boli"/>
+        <a:font script="Deva" typeface="Mangal"/>
+        <a:font script="Telu" typeface="Gautami"/>
+        <a:font script="Taml" typeface="Latha"/>
+        <a:font script="Syrc" typeface="Estrangelo Edessa"/>
+        <a:font script="Orya" typeface="Kalinga"/>
+        <a:font script="Mlym" typeface="Kartika"/>
+        <a:font script="Laoo" typeface="DokChampa"/>
+        <a:font script="Sinh" typeface="Iskoola Pota"/>
+        <a:font script="Mong" typeface="Mongolian Baiti"/>
+        <a:font script="Viet" typeface="Arial"/>
+        <a:font script="Uigh" typeface="Microsoft Uighur"/>
+        <a:font script="Geor" typeface="Sylfaen"/>
       </a:minorFont>
     </a:fontScheme>
     <a:fmtScheme name="Office">
@@ -470,7 +477,7 @@
               </a:schemeClr>
             </a:gs>
           </a:gsLst>
-          <a:lin scaled="1" ang="16200000"/>
+          <a:lin ang="16200000" scaled="1"/>
         </a:gradFill>
         <a:gradFill rotWithShape="1">
           <a:gsLst>
@@ -493,11 +500,11 @@
               </a:schemeClr>
             </a:gs>
           </a:gsLst>
-          <a:lin scaled="1" ang="16200000"/>
+          <a:lin ang="16200000" scaled="1"/>
         </a:gradFill>
       </a:fillStyleLst>
       <a:lnStyleLst>
-        <a:ln algn="ctr" cmpd="sng" cap="flat" w="9525">
+        <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
           <a:solidFill>
             <a:schemeClr val="phClr">
               <a:shade val="9500"/>
@@ -506,13 +513,13 @@
           </a:solidFill>
           <a:prstDash val="solid"/>
         </a:ln>
-        <a:ln algn="ctr" cmpd="sng" cap="flat" w="25400">
+        <a:ln w="25400" cap="flat" cmpd="sng" algn="ctr">
           <a:solidFill>
             <a:schemeClr val="phClr"/>
           </a:solidFill>
           <a:prstDash val="solid"/>
         </a:ln>
-        <a:ln algn="ctr" cmpd="sng" cap="flat" w="38100">
+        <a:ln w="38100" cap="flat" cmpd="sng" algn="ctr">
           <a:solidFill>
             <a:schemeClr val="phClr"/>
           </a:solidFill>
@@ -522,7 +529,7 @@
       <a:effectStyleLst>
         <a:effectStyle>
           <a:effectLst>
-            <a:outerShdw dir="5400000" rotWithShape="0" dist="23000" blurRad="40000">
+            <a:outerShdw blurRad="40000" dist="23000" dir="5400000" rotWithShape="0">
               <a:srgbClr val="000000">
                 <a:alpha val="38000"/>
               </a:srgbClr>
@@ -531,7 +538,7 @@
         </a:effectStyle>
         <a:effectStyle>
           <a:effectLst>
-            <a:outerShdw dir="5400000" rotWithShape="0" dist="23000" blurRad="40000">
+            <a:outerShdw blurRad="40000" dist="23000" dir="5400000" rotWithShape="0">
               <a:srgbClr val="000000">
                 <a:alpha val="35000"/>
               </a:srgbClr>
@@ -540,7 +547,7 @@
         </a:effectStyle>
         <a:effectStyle>
           <a:effectLst>
-            <a:outerShdw dir="5400000" rotWithShape="0" dist="23000" blurRad="40000">
+            <a:outerShdw blurRad="40000" dist="23000" dir="5400000" rotWithShape="0">
               <a:srgbClr val="000000">
                 <a:alpha val="35000"/>
               </a:srgbClr>
@@ -548,10 +555,10 @@
           </a:effectLst>
           <a:scene3d>
             <a:camera prst="orthographicFront">
-              <a:rot rev="0" lon="0" lat="0"/>
+              <a:rot lat="0" lon="0" rev="0"/>
             </a:camera>
-            <a:lightRig dir="t" rig="threePt">
-              <a:rot rev="1200000" lon="0" lat="0"/>
+            <a:lightRig rig="threePt" dir="t">
+              <a:rot lat="0" lon="0" rev="1200000"/>
             </a:lightRig>
           </a:scene3d>
           <a:sp3d>
@@ -621,23 +628,23 @@
     <outlinePr summaryBelow="0"/>
   </sheetPr>
   <dimension ref="A1:B13"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" style="2" width="30.719285714285714" customWidth="1" bestFit="1"/>
-    <col min="2" max="2" style="12" width="20.719285714285714" customWidth="1" bestFit="1"/>
+    <col min="1" max="1" width="30.6640625" style="2" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="20.6640625" style="12" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row x14ac:dyDescent="0.25" r="1" customHeight="1" ht="18.75">
-      <c r="A1" s="3" t="s">
+    <row r="1" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A1" s="13" t="s">
         <v>43</v>
       </c>
-      <c r="B1" s="4"/>
-    </row>
-    <row x14ac:dyDescent="0.25" r="2" customHeight="1" ht="18.75">
+      <c r="B1" s="14"/>
+    </row>
+    <row r="2" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A2" s="1"/>
       <c r="B2" s="10"/>
     </row>
-    <row x14ac:dyDescent="0.25" r="3" customHeight="1" ht="18.75">
+    <row r="3" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="1" t="s">
         <v>44</v>
       </c>
@@ -645,17 +652,17 @@
         <v>45</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="4" customHeight="1" ht="18.75">
+    <row r="4" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A4" s="1"/>
       <c r="B4" s="10"/>
     </row>
-    <row x14ac:dyDescent="0.25" r="5" customHeight="1" ht="18.75">
-      <c r="A5" s="3" t="s">
+    <row r="5" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A5" s="13" t="s">
         <v>46</v>
       </c>
-      <c r="B5" s="4"/>
-    </row>
-    <row x14ac:dyDescent="0.25" r="6" customHeight="1" ht="18.75">
+      <c r="B5" s="14"/>
+    </row>
+    <row r="6" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A6" s="1" t="s">
         <v>47</v>
       </c>
@@ -663,7 +670,7 @@
         <v>2</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="7" customHeight="1" ht="18.75">
+    <row r="7" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A7" s="1" t="s">
         <v>48</v>
       </c>
@@ -671,7 +678,7 @@
         <v>6</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="8" customHeight="1" ht="18.75">
+    <row r="8" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A8" s="1" t="s">
         <v>49</v>
       </c>
@@ -679,41 +686,41 @@
         <v>8</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="9" customHeight="1" ht="18.75">
+    <row r="9" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A9" s="1"/>
       <c r="B9" s="10"/>
     </row>
-    <row x14ac:dyDescent="0.25" r="10" customHeight="1" ht="18.75">
-      <c r="A10" s="3" t="s">
+    <row r="10" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A10" s="13" t="s">
         <v>50</v>
       </c>
-      <c r="B10" s="4"/>
-    </row>
-    <row x14ac:dyDescent="0.25" r="11" customHeight="1" ht="18.75">
+      <c r="B10" s="14"/>
+    </row>
+    <row r="11" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A11" s="1" t="s">
         <v>51</v>
       </c>
       <c r="B11" s="7">
         <f>B3+(B6*7)</f>
-        <v>25568.875</v>
-      </c>
-    </row>
-    <row x14ac:dyDescent="0.25" r="12" customHeight="1" ht="18.75">
+        <v>46119</v>
+      </c>
+    </row>
+    <row r="12" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A12" s="1" t="s">
         <v>52</v>
       </c>
       <c r="B12" s="7">
         <f>B11+(B7*7)</f>
-        <v>25568.875</v>
-      </c>
-    </row>
-    <row x14ac:dyDescent="0.25" r="13" customHeight="1" ht="18.75">
+        <v>46161</v>
+      </c>
+    </row>
+    <row r="13" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A13" s="1" t="s">
         <v>53</v>
       </c>
       <c r="B13" s="7">
         <f>B12+(B8*7)</f>
-        <v>25568.875</v>
+        <v>46217</v>
       </c>
     </row>
   </sheetData>
@@ -732,16 +739,16 @@
     <outlinePr summaryBelow="0"/>
   </sheetPr>
   <dimension ref="A1:E21"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" style="9" width="15.719285714285713" customWidth="1" bestFit="1"/>
-    <col min="2" max="2" style="2" width="15.719285714285713" customWidth="1" bestFit="1"/>
-    <col min="3" max="3" style="6" width="20.719285714285714" customWidth="1" bestFit="1"/>
-    <col min="4" max="4" style="6" width="40.71928571428572" customWidth="1" bestFit="1"/>
-    <col min="5" max="5" style="2" width="15.719285714285713" customWidth="1" bestFit="1"/>
+    <col min="1" max="1" width="15.6640625" style="9" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="15.6640625" style="2" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="20.6640625" style="6" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="40.6640625" style="6" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="15.6640625" style="2" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row x14ac:dyDescent="0.25" r="1" customHeight="1" ht="18.75">
+    <row r="1" spans="1:5" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A1" s="3" t="s">
         <v>17</v>
       </c>
@@ -758,361 +765,401 @@
         <v>21</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="2" customHeight="1" ht="18.75">
+    <row r="2" spans="1:5" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A2" s="7">
         <f>'Configuração Inicial'!$B$3+(1-1)*7</f>
-        <v>25568.875</v>
+        <v>46105</v>
       </c>
       <c r="B2" s="1" t="s">
         <v>22</v>
       </c>
-      <c r="C2" s="8">
+      <c r="C2" s="8" t="str">
         <f>IF(1&lt;='Configuração Inicial'!$B$6, "Clone", IF(1&lt;='Configuração Inicial'!$B$6+'Configuração Inicial'!$B$7, "Vegetativo", "Floração"))</f>
-      </c>
-      <c r="D2" s="8">
-        <f>IF(C2="Clone", "Umidade Alta (70%), Luz Suave", IF(C2="Vegetativo", "Nitrogênio Alto, LST/Poda", IF(C2="Floração", "Fósforo/Potássio, Reduzir Umidade", "Aguardar")))</f>
+        <v>Clone</v>
+      </c>
+      <c r="D2" s="8" t="str">
+        <f t="shared" ref="D2:D21" si="0">IF(C2="Clone", "Umidade Alta (70%), Luz Suave", IF(C2="Vegetativo", "Nitrogênio Alto, LST/Poda", IF(C2="Floração", "Fósforo/Potássio, Reduzir Umidade", "Aguardar")))</f>
+        <v>Umidade Alta (70%), Luz Suave</v>
       </c>
       <c r="E2" s="1" t="s">
         <v>23</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="3" customHeight="1" ht="18.75">
+    <row r="3" spans="1:5" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="7">
         <f>'Configuração Inicial'!$B$3+(2-1)*7</f>
-        <v>25568.875</v>
+        <v>46112</v>
       </c>
       <c r="B3" s="1" t="s">
         <v>24</v>
       </c>
-      <c r="C3" s="8">
+      <c r="C3" s="8" t="str">
         <f>IF(2&lt;='Configuração Inicial'!$B$6, "Clone", IF(2&lt;='Configuração Inicial'!$B$6+'Configuração Inicial'!$B$7, "Vegetativo", "Floração"))</f>
-      </c>
-      <c r="D3" s="8">
-        <f>IF(C3="Clone", "Umidade Alta (70%), Luz Suave", IF(C3="Vegetativo", "Nitrogênio Alto, LST/Poda", IF(C3="Floração", "Fósforo/Potássio, Reduzir Umidade", "Aguardar")))</f>
+        <v>Clone</v>
+      </c>
+      <c r="D3" s="8" t="str">
+        <f t="shared" si="0"/>
+        <v>Umidade Alta (70%), Luz Suave</v>
       </c>
       <c r="E3" s="1" t="s">
         <v>23</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="4" customHeight="1" ht="18.75">
+    <row r="4" spans="1:5" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A4" s="7">
         <f>'Configuração Inicial'!$B$3+(3-1)*7</f>
-        <v>25568.875</v>
+        <v>46119</v>
       </c>
       <c r="B4" s="1" t="s">
         <v>25</v>
       </c>
-      <c r="C4" s="8">
+      <c r="C4" s="8" t="str">
         <f>IF(3&lt;='Configuração Inicial'!$B$6, "Clone", IF(3&lt;='Configuração Inicial'!$B$6+'Configuração Inicial'!$B$7, "Vegetativo", "Floração"))</f>
-      </c>
-      <c r="D4" s="8">
-        <f>IF(C4="Clone", "Umidade Alta (70%), Luz Suave", IF(C4="Vegetativo", "Nitrogênio Alto, LST/Poda", IF(C4="Floração", "Fósforo/Potássio, Reduzir Umidade", "Aguardar")))</f>
+        <v>Vegetativo</v>
+      </c>
+      <c r="D4" s="8" t="str">
+        <f t="shared" si="0"/>
+        <v>Nitrogênio Alto, LST/Poda</v>
       </c>
       <c r="E4" s="1" t="s">
         <v>23</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="5" customHeight="1" ht="18.75">
+    <row r="5" spans="1:5" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A5" s="7">
         <f>'Configuração Inicial'!$B$3+(4-1)*7</f>
-        <v>25568.875</v>
+        <v>46126</v>
       </c>
       <c r="B5" s="1" t="s">
         <v>26</v>
       </c>
-      <c r="C5" s="8">
+      <c r="C5" s="8" t="str">
         <f>IF(4&lt;='Configuração Inicial'!$B$6, "Clone", IF(4&lt;='Configuração Inicial'!$B$6+'Configuração Inicial'!$B$7, "Vegetativo", "Floração"))</f>
-      </c>
-      <c r="D5" s="8">
-        <f>IF(C5="Clone", "Umidade Alta (70%), Luz Suave", IF(C5="Vegetativo", "Nitrogênio Alto, LST/Poda", IF(C5="Floração", "Fósforo/Potássio, Reduzir Umidade", "Aguardar")))</f>
+        <v>Vegetativo</v>
+      </c>
+      <c r="D5" s="8" t="str">
+        <f t="shared" si="0"/>
+        <v>Nitrogênio Alto, LST/Poda</v>
       </c>
       <c r="E5" s="1" t="s">
         <v>23</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="6" customHeight="1" ht="18.75">
+    <row r="6" spans="1:5" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A6" s="7">
         <f>'Configuração Inicial'!$B$3+(5-1)*7</f>
-        <v>25568.875</v>
+        <v>46133</v>
       </c>
       <c r="B6" s="1" t="s">
         <v>27</v>
       </c>
-      <c r="C6" s="8">
+      <c r="C6" s="8" t="str">
         <f>IF(5&lt;='Configuração Inicial'!$B$6, "Clone", IF(5&lt;='Configuração Inicial'!$B$6+'Configuração Inicial'!$B$7, "Vegetativo", "Floração"))</f>
-      </c>
-      <c r="D6" s="8">
-        <f>IF(C6="Clone", "Umidade Alta (70%), Luz Suave", IF(C6="Vegetativo", "Nitrogênio Alto, LST/Poda", IF(C6="Floração", "Fósforo/Potássio, Reduzir Umidade", "Aguardar")))</f>
+        <v>Vegetativo</v>
+      </c>
+      <c r="D6" s="8" t="str">
+        <f t="shared" si="0"/>
+        <v>Nitrogênio Alto, LST/Poda</v>
       </c>
       <c r="E6" s="1" t="s">
         <v>23</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="7" customHeight="1" ht="18.75">
+    <row r="7" spans="1:5" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A7" s="7">
         <f>'Configuração Inicial'!$B$3+(6-1)*7</f>
-        <v>25568.875</v>
+        <v>46140</v>
       </c>
       <c r="B7" s="1" t="s">
         <v>28</v>
       </c>
-      <c r="C7" s="8">
+      <c r="C7" s="8" t="str">
         <f>IF(6&lt;='Configuração Inicial'!$B$6, "Clone", IF(6&lt;='Configuração Inicial'!$B$6+'Configuração Inicial'!$B$7, "Vegetativo", "Floração"))</f>
-      </c>
-      <c r="D7" s="8">
-        <f>IF(C7="Clone", "Umidade Alta (70%), Luz Suave", IF(C7="Vegetativo", "Nitrogênio Alto, LST/Poda", IF(C7="Floração", "Fósforo/Potássio, Reduzir Umidade", "Aguardar")))</f>
+        <v>Vegetativo</v>
+      </c>
+      <c r="D7" s="8" t="str">
+        <f t="shared" si="0"/>
+        <v>Nitrogênio Alto, LST/Poda</v>
       </c>
       <c r="E7" s="1" t="s">
         <v>23</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="8" customHeight="1" ht="18.75">
+    <row r="8" spans="1:5" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A8" s="7">
         <f>'Configuração Inicial'!$B$3+(7-1)*7</f>
-        <v>25568.875</v>
+        <v>46147</v>
       </c>
       <c r="B8" s="1" t="s">
         <v>29</v>
       </c>
-      <c r="C8" s="8">
+      <c r="C8" s="8" t="str">
         <f>IF(7&lt;='Configuração Inicial'!$B$6, "Clone", IF(7&lt;='Configuração Inicial'!$B$6+'Configuração Inicial'!$B$7, "Vegetativo", "Floração"))</f>
-      </c>
-      <c r="D8" s="8">
-        <f>IF(C8="Clone", "Umidade Alta (70%), Luz Suave", IF(C8="Vegetativo", "Nitrogênio Alto, LST/Poda", IF(C8="Floração", "Fósforo/Potássio, Reduzir Umidade", "Aguardar")))</f>
+        <v>Vegetativo</v>
+      </c>
+      <c r="D8" s="8" t="str">
+        <f t="shared" si="0"/>
+        <v>Nitrogênio Alto, LST/Poda</v>
       </c>
       <c r="E8" s="1" t="s">
         <v>23</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="9" customHeight="1" ht="18.75">
+    <row r="9" spans="1:5" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A9" s="7">
         <f>'Configuração Inicial'!$B$3+(8-1)*7</f>
-        <v>25568.875</v>
+        <v>46154</v>
       </c>
       <c r="B9" s="1" t="s">
         <v>30</v>
       </c>
-      <c r="C9" s="8">
+      <c r="C9" s="8" t="str">
         <f>IF(8&lt;='Configuração Inicial'!$B$6, "Clone", IF(8&lt;='Configuração Inicial'!$B$6+'Configuração Inicial'!$B$7, "Vegetativo", "Floração"))</f>
-      </c>
-      <c r="D9" s="8">
-        <f>IF(C9="Clone", "Umidade Alta (70%), Luz Suave", IF(C9="Vegetativo", "Nitrogênio Alto, LST/Poda", IF(C9="Floração", "Fósforo/Potássio, Reduzir Umidade", "Aguardar")))</f>
+        <v>Vegetativo</v>
+      </c>
+      <c r="D9" s="8" t="str">
+        <f t="shared" si="0"/>
+        <v>Nitrogênio Alto, LST/Poda</v>
       </c>
       <c r="E9" s="1" t="s">
         <v>23</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="10" customHeight="1" ht="18.75">
+    <row r="10" spans="1:5" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A10" s="7">
         <f>'Configuração Inicial'!$B$3+(9-1)*7</f>
-        <v>25568.875</v>
+        <v>46161</v>
       </c>
       <c r="B10" s="1" t="s">
         <v>31</v>
       </c>
-      <c r="C10" s="8">
+      <c r="C10" s="8" t="str">
         <f>IF(9&lt;='Configuração Inicial'!$B$6, "Clone", IF(9&lt;='Configuração Inicial'!$B$6+'Configuração Inicial'!$B$7, "Vegetativo", "Floração"))</f>
-      </c>
-      <c r="D10" s="8">
-        <f>IF(C10="Clone", "Umidade Alta (70%), Luz Suave", IF(C10="Vegetativo", "Nitrogênio Alto, LST/Poda", IF(C10="Floração", "Fósforo/Potássio, Reduzir Umidade", "Aguardar")))</f>
+        <v>Floração</v>
+      </c>
+      <c r="D10" s="8" t="str">
+        <f t="shared" si="0"/>
+        <v>Fósforo/Potássio, Reduzir Umidade</v>
       </c>
       <c r="E10" s="1" t="s">
         <v>23</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="11" customHeight="1" ht="18.75">
+    <row r="11" spans="1:5" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A11" s="7">
         <f>'Configuração Inicial'!$B$3+(10-1)*7</f>
-        <v>25568.875</v>
+        <v>46168</v>
       </c>
       <c r="B11" s="1" t="s">
         <v>32</v>
       </c>
-      <c r="C11" s="8">
+      <c r="C11" s="8" t="str">
         <f>IF(10&lt;='Configuração Inicial'!$B$6, "Clone", IF(10&lt;='Configuração Inicial'!$B$6+'Configuração Inicial'!$B$7, "Vegetativo", "Floração"))</f>
-      </c>
-      <c r="D11" s="8">
-        <f>IF(C11="Clone", "Umidade Alta (70%), Luz Suave", IF(C11="Vegetativo", "Nitrogênio Alto, LST/Poda", IF(C11="Floração", "Fósforo/Potássio, Reduzir Umidade", "Aguardar")))</f>
+        <v>Floração</v>
+      </c>
+      <c r="D11" s="8" t="str">
+        <f t="shared" si="0"/>
+        <v>Fósforo/Potássio, Reduzir Umidade</v>
       </c>
       <c r="E11" s="1" t="s">
         <v>23</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="12" customHeight="1" ht="18.75">
+    <row r="12" spans="1:5" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A12" s="7">
         <f>'Configuração Inicial'!$B$3+(11-1)*7</f>
-        <v>25568.875</v>
+        <v>46175</v>
       </c>
       <c r="B12" s="1" t="s">
         <v>33</v>
       </c>
-      <c r="C12" s="8">
+      <c r="C12" s="8" t="str">
         <f>IF(11&lt;='Configuração Inicial'!$B$6, "Clone", IF(11&lt;='Configuração Inicial'!$B$6+'Configuração Inicial'!$B$7, "Vegetativo", "Floração"))</f>
-      </c>
-      <c r="D12" s="8">
-        <f>IF(C12="Clone", "Umidade Alta (70%), Luz Suave", IF(C12="Vegetativo", "Nitrogênio Alto, LST/Poda", IF(C12="Floração", "Fósforo/Potássio, Reduzir Umidade", "Aguardar")))</f>
+        <v>Floração</v>
+      </c>
+      <c r="D12" s="8" t="str">
+        <f t="shared" si="0"/>
+        <v>Fósforo/Potássio, Reduzir Umidade</v>
       </c>
       <c r="E12" s="1" t="s">
         <v>23</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="13" customHeight="1" ht="18.75">
+    <row r="13" spans="1:5" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A13" s="7">
         <f>'Configuração Inicial'!$B$3+(12-1)*7</f>
-        <v>25568.875</v>
+        <v>46182</v>
       </c>
       <c r="B13" s="1" t="s">
         <v>34</v>
       </c>
-      <c r="C13" s="8">
+      <c r="C13" s="8" t="str">
         <f>IF(12&lt;='Configuração Inicial'!$B$6, "Clone", IF(12&lt;='Configuração Inicial'!$B$6+'Configuração Inicial'!$B$7, "Vegetativo", "Floração"))</f>
-      </c>
-      <c r="D13" s="8">
-        <f>IF(C13="Clone", "Umidade Alta (70%), Luz Suave", IF(C13="Vegetativo", "Nitrogênio Alto, LST/Poda", IF(C13="Floração", "Fósforo/Potássio, Reduzir Umidade", "Aguardar")))</f>
+        <v>Floração</v>
+      </c>
+      <c r="D13" s="8" t="str">
+        <f t="shared" si="0"/>
+        <v>Fósforo/Potássio, Reduzir Umidade</v>
       </c>
       <c r="E13" s="1" t="s">
         <v>23</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="14" customHeight="1" ht="18.75">
+    <row r="14" spans="1:5" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A14" s="7">
         <f>'Configuração Inicial'!$B$3+(13-1)*7</f>
-        <v>25568.875</v>
+        <v>46189</v>
       </c>
       <c r="B14" s="1" t="s">
         <v>35</v>
       </c>
-      <c r="C14" s="8">
+      <c r="C14" s="8" t="str">
         <f>IF(13&lt;='Configuração Inicial'!$B$6, "Clone", IF(13&lt;='Configuração Inicial'!$B$6+'Configuração Inicial'!$B$7, "Vegetativo", "Floração"))</f>
-      </c>
-      <c r="D14" s="8">
-        <f>IF(C14="Clone", "Umidade Alta (70%), Luz Suave", IF(C14="Vegetativo", "Nitrogênio Alto, LST/Poda", IF(C14="Floração", "Fósforo/Potássio, Reduzir Umidade", "Aguardar")))</f>
+        <v>Floração</v>
+      </c>
+      <c r="D14" s="8" t="str">
+        <f t="shared" si="0"/>
+        <v>Fósforo/Potássio, Reduzir Umidade</v>
       </c>
       <c r="E14" s="1" t="s">
         <v>23</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="15" customHeight="1" ht="18.75">
+    <row r="15" spans="1:5" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A15" s="7">
         <f>'Configuração Inicial'!$B$3+(14-1)*7</f>
-        <v>25568.875</v>
+        <v>46196</v>
       </c>
       <c r="B15" s="1" t="s">
         <v>36</v>
       </c>
-      <c r="C15" s="8">
+      <c r="C15" s="8" t="str">
         <f>IF(14&lt;='Configuração Inicial'!$B$6, "Clone", IF(14&lt;='Configuração Inicial'!$B$6+'Configuração Inicial'!$B$7, "Vegetativo", "Floração"))</f>
-      </c>
-      <c r="D15" s="8">
-        <f>IF(C15="Clone", "Umidade Alta (70%), Luz Suave", IF(C15="Vegetativo", "Nitrogênio Alto, LST/Poda", IF(C15="Floração", "Fósforo/Potássio, Reduzir Umidade", "Aguardar")))</f>
+        <v>Floração</v>
+      </c>
+      <c r="D15" s="8" t="str">
+        <f t="shared" si="0"/>
+        <v>Fósforo/Potássio, Reduzir Umidade</v>
       </c>
       <c r="E15" s="1" t="s">
         <v>23</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="16" customHeight="1" ht="18.75">
+    <row r="16" spans="1:5" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A16" s="7">
         <f>'Configuração Inicial'!$B$3+(15-1)*7</f>
-        <v>25568.875</v>
+        <v>46203</v>
       </c>
       <c r="B16" s="1" t="s">
         <v>37</v>
       </c>
-      <c r="C16" s="8">
+      <c r="C16" s="8" t="str">
         <f>IF(15&lt;='Configuração Inicial'!$B$6, "Clone", IF(15&lt;='Configuração Inicial'!$B$6+'Configuração Inicial'!$B$7, "Vegetativo", "Floração"))</f>
-      </c>
-      <c r="D16" s="8">
-        <f>IF(C16="Clone", "Umidade Alta (70%), Luz Suave", IF(C16="Vegetativo", "Nitrogênio Alto, LST/Poda", IF(C16="Floração", "Fósforo/Potássio, Reduzir Umidade", "Aguardar")))</f>
+        <v>Floração</v>
+      </c>
+      <c r="D16" s="8" t="str">
+        <f t="shared" si="0"/>
+        <v>Fósforo/Potássio, Reduzir Umidade</v>
       </c>
       <c r="E16" s="1" t="s">
         <v>23</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="17" customHeight="1" ht="18.75">
+    <row r="17" spans="1:5" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A17" s="7">
         <f>'Configuração Inicial'!$B$3+(16-1)*7</f>
-        <v>25568.875</v>
+        <v>46210</v>
       </c>
       <c r="B17" s="1" t="s">
         <v>38</v>
       </c>
-      <c r="C17" s="8">
+      <c r="C17" s="8" t="str">
         <f>IF(16&lt;='Configuração Inicial'!$B$6, "Clone", IF(16&lt;='Configuração Inicial'!$B$6+'Configuração Inicial'!$B$7, "Vegetativo", "Floração"))</f>
-      </c>
-      <c r="D17" s="8">
-        <f>IF(C17="Clone", "Umidade Alta (70%), Luz Suave", IF(C17="Vegetativo", "Nitrogênio Alto, LST/Poda", IF(C17="Floração", "Fósforo/Potássio, Reduzir Umidade", "Aguardar")))</f>
+        <v>Floração</v>
+      </c>
+      <c r="D17" s="8" t="str">
+        <f t="shared" si="0"/>
+        <v>Fósforo/Potássio, Reduzir Umidade</v>
       </c>
       <c r="E17" s="1" t="s">
         <v>23</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="18" customHeight="1" ht="18.75">
+    <row r="18" spans="1:5" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A18" s="7">
         <f>'Configuração Inicial'!$B$3+(17-1)*7</f>
-        <v>25568.875</v>
+        <v>46217</v>
       </c>
       <c r="B18" s="1" t="s">
         <v>39</v>
       </c>
-      <c r="C18" s="8">
+      <c r="C18" s="8" t="str">
         <f>IF(17&lt;='Configuração Inicial'!$B$6, "Clone", IF(17&lt;='Configuração Inicial'!$B$6+'Configuração Inicial'!$B$7, "Vegetativo", "Floração"))</f>
-      </c>
-      <c r="D18" s="8">
-        <f>IF(C18="Clone", "Umidade Alta (70%), Luz Suave", IF(C18="Vegetativo", "Nitrogênio Alto, LST/Poda", IF(C18="Floração", "Fósforo/Potássio, Reduzir Umidade", "Aguardar")))</f>
+        <v>Floração</v>
+      </c>
+      <c r="D18" s="8" t="str">
+        <f t="shared" si="0"/>
+        <v>Fósforo/Potássio, Reduzir Umidade</v>
       </c>
       <c r="E18" s="1" t="s">
         <v>23</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="19" customHeight="1" ht="18.75">
+    <row r="19" spans="1:5" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A19" s="7">
         <f>'Configuração Inicial'!$B$3+(18-1)*7</f>
-        <v>25568.875</v>
+        <v>46224</v>
       </c>
       <c r="B19" s="1" t="s">
         <v>40</v>
       </c>
-      <c r="C19" s="8">
+      <c r="C19" s="8" t="str">
         <f>IF(18&lt;='Configuração Inicial'!$B$6, "Clone", IF(18&lt;='Configuração Inicial'!$B$6+'Configuração Inicial'!$B$7, "Vegetativo", "Floração"))</f>
-      </c>
-      <c r="D19" s="8">
-        <f>IF(C19="Clone", "Umidade Alta (70%), Luz Suave", IF(C19="Vegetativo", "Nitrogênio Alto, LST/Poda", IF(C19="Floração", "Fósforo/Potássio, Reduzir Umidade", "Aguardar")))</f>
+        <v>Floração</v>
+      </c>
+      <c r="D19" s="8" t="str">
+        <f t="shared" si="0"/>
+        <v>Fósforo/Potássio, Reduzir Umidade</v>
       </c>
       <c r="E19" s="1" t="s">
         <v>23</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="20" customHeight="1" ht="18.75">
+    <row r="20" spans="1:5" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A20" s="7">
         <f>'Configuração Inicial'!$B$3+(19-1)*7</f>
-        <v>25568.875</v>
+        <v>46231</v>
       </c>
       <c r="B20" s="1" t="s">
         <v>41</v>
       </c>
-      <c r="C20" s="8">
+      <c r="C20" s="8" t="str">
         <f>IF(19&lt;='Configuração Inicial'!$B$6, "Clone", IF(19&lt;='Configuração Inicial'!$B$6+'Configuração Inicial'!$B$7, "Vegetativo", "Floração"))</f>
-      </c>
-      <c r="D20" s="8">
-        <f>IF(C20="Clone", "Umidade Alta (70%), Luz Suave", IF(C20="Vegetativo", "Nitrogênio Alto, LST/Poda", IF(C20="Floração", "Fósforo/Potássio, Reduzir Umidade", "Aguardar")))</f>
+        <v>Floração</v>
+      </c>
+      <c r="D20" s="8" t="str">
+        <f t="shared" si="0"/>
+        <v>Fósforo/Potássio, Reduzir Umidade</v>
       </c>
       <c r="E20" s="1" t="s">
         <v>23</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="21" customHeight="1" ht="18.75">
+    <row r="21" spans="1:5" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A21" s="7">
         <f>'Configuração Inicial'!$B$3+(20-1)*7</f>
-        <v>25568.875</v>
+        <v>46238</v>
       </c>
       <c r="B21" s="1" t="s">
         <v>42</v>
       </c>
-      <c r="C21" s="8">
+      <c r="C21" s="8" t="str">
         <f>IF(20&lt;='Configuração Inicial'!$B$6, "Clone", IF(20&lt;='Configuração Inicial'!$B$6+'Configuração Inicial'!$B$7, "Vegetativo", "Floração"))</f>
-      </c>
-      <c r="D21" s="8">
-        <f>IF(C21="Clone", "Umidade Alta (70%), Luz Suave", IF(C21="Vegetativo", "Nitrogênio Alto, LST/Poda", IF(C21="Floração", "Fósforo/Potássio, Reduzir Umidade", "Aguardar")))</f>
+        <v>Floração</v>
+      </c>
+      <c r="D21" s="8" t="str">
+        <f t="shared" si="0"/>
+        <v>Fósforo/Potássio, Reduzir Umidade</v>
       </c>
       <c r="E21" s="1" t="s">
         <v>23</v>
@@ -1129,15 +1176,15 @@
     <outlinePr summaryBelow="0"/>
   </sheetPr>
   <dimension ref="A1:D11"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" style="2" width="15.719285714285713" customWidth="1" bestFit="1"/>
-    <col min="2" max="2" style="2" width="20.719285714285714" customWidth="1" bestFit="1"/>
-    <col min="3" max="3" style="6" width="50.71928571428572" customWidth="1" bestFit="1"/>
-    <col min="4" max="4" style="2" width="20.719285714285714" customWidth="1" bestFit="1"/>
+    <col min="1" max="1" width="15.6640625" style="2" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="20.6640625" style="2" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="50.6640625" style="6" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="20.6640625" style="2" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row x14ac:dyDescent="0.25" r="1" customHeight="1" ht="20.25">
+    <row r="1" spans="1:4" ht="20.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A1" s="3" t="s">
         <v>12</v>
       </c>
@@ -1151,121 +1198,131 @@
         <v>15</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="2" customHeight="1" ht="19.5">
+    <row r="2" spans="1:4" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A2" s="1"/>
       <c r="B2" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="C2" s="5">
+      <c r="C2" s="5" t="str">
         <f>VLOOKUP(B2, Database!$A$1:$B$6, 2, FALSE)</f>
+        <v>Manter monitoramento preventivo</v>
       </c>
       <c r="D2" s="1" t="s">
         <v>16</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="3" customHeight="1" ht="19.5">
+    <row r="3" spans="1:4" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="1"/>
       <c r="B3" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="C3" s="5">
+      <c r="C3" s="5" t="str">
         <f>VLOOKUP(B3, Database!$A$1:$B$6, 2, FALSE)</f>
+        <v>Manter monitoramento preventivo</v>
       </c>
       <c r="D3" s="1" t="s">
         <v>16</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="4" customHeight="1" ht="19.5">
+    <row r="4" spans="1:4" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A4" s="1"/>
       <c r="B4" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="C4" s="5">
+      <c r="C4" s="5" t="str">
         <f>VLOOKUP(B4, Database!$A$1:$B$6, 2, FALSE)</f>
+        <v>Manter monitoramento preventivo</v>
       </c>
       <c r="D4" s="1" t="s">
         <v>16</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="5" customHeight="1" ht="19.5">
+    <row r="5" spans="1:4" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A5" s="1"/>
       <c r="B5" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="C5" s="5">
+      <c r="C5" s="5" t="str">
         <f>VLOOKUP(B5, Database!$A$1:$B$6, 2, FALSE)</f>
+        <v>Manter monitoramento preventivo</v>
       </c>
       <c r="D5" s="1" t="s">
         <v>16</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="6" customHeight="1" ht="19.5">
+    <row r="6" spans="1:4" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A6" s="1"/>
       <c r="B6" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="C6" s="5">
+      <c r="C6" s="5" t="str">
         <f>VLOOKUP(B6, Database!$A$1:$B$6, 2, FALSE)</f>
+        <v>Manter monitoramento preventivo</v>
       </c>
       <c r="D6" s="1" t="s">
         <v>16</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="7" customHeight="1" ht="19.5">
+    <row r="7" spans="1:4" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A7" s="1"/>
       <c r="B7" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="C7" s="5">
+      <c r="C7" s="5" t="str">
         <f>VLOOKUP(B7, Database!$A$1:$B$6, 2, FALSE)</f>
+        <v>Manter monitoramento preventivo</v>
       </c>
       <c r="D7" s="1" t="s">
         <v>16</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="8" customHeight="1" ht="19.5">
+    <row r="8" spans="1:4" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A8" s="1"/>
       <c r="B8" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="C8" s="5">
+      <c r="C8" s="5" t="str">
         <f>VLOOKUP(B8, Database!$A$1:$B$6, 2, FALSE)</f>
+        <v>Manter monitoramento preventivo</v>
       </c>
       <c r="D8" s="1" t="s">
         <v>16</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="9" customHeight="1" ht="19.5">
+    <row r="9" spans="1:4" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A9" s="1"/>
       <c r="B9" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="C9" s="5">
+      <c r="C9" s="5" t="str">
         <f>VLOOKUP(B9, Database!$A$1:$B$6, 2, FALSE)</f>
+        <v>Manter monitoramento preventivo</v>
       </c>
       <c r="D9" s="1" t="s">
         <v>16</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="10" customHeight="1" ht="19.5">
+    <row r="10" spans="1:4" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A10" s="1"/>
       <c r="B10" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="C10" s="5">
+      <c r="C10" s="5" t="str">
         <f>VLOOKUP(B10, Database!$A$1:$B$6, 2, FALSE)</f>
+        <v>Manter monitoramento preventivo</v>
       </c>
       <c r="D10" s="1" t="s">
         <v>16</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="11" customHeight="1" ht="20.25">
+    <row r="11" spans="1:4" ht="20.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A11" s="1"/>
       <c r="B11" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="C11" s="5">
+      <c r="C11" s="5" t="str">
         <f>VLOOKUP(B11, Database!$A$1:$B$6, 2, FALSE)</f>
+        <v>Manter monitoramento preventivo</v>
       </c>
       <c r="D11" s="1" t="s">
         <v>16</v>
@@ -1282,13 +1339,12 @@
     <outlinePr summaryBelow="0"/>
   </sheetPr>
   <dimension ref="A1:B6"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" style="2" width="13.576428571428572" customWidth="1" bestFit="1"/>
-    <col min="2" max="2" style="2" width="13.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="1" max="2" width="13.5546875" style="2" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row x14ac:dyDescent="0.25" r="1" customHeight="1" ht="18.75">
+    <row r="1" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1296,7 +1352,7 @@
         <v>1</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="2" customHeight="1" ht="18.75">
+    <row r="2" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A2" s="1" t="s">
         <v>2</v>
       </c>
@@ -1304,7 +1360,7 @@
         <v>3</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="3" customHeight="1" ht="18.75">
+    <row r="3" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="1" t="s">
         <v>4</v>
       </c>
@@ -1312,7 +1368,7 @@
         <v>5</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="4" customHeight="1" ht="18.75">
+    <row r="4" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A4" s="1" t="s">
         <v>6</v>
       </c>
@@ -1320,7 +1376,7 @@
         <v>7</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="5" customHeight="1" ht="18.75">
+    <row r="5" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A5" s="1" t="s">
         <v>8</v>
       </c>
@@ -1328,7 +1384,7 @@
         <v>9</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="6" customHeight="1" ht="18.75">
+    <row r="6" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A6" s="1" t="s">
         <v>10</v>
       </c>

</xml_diff>